<commit_message>
Gästeportal Englisch: Korrekturen aus dem Gegenlesen übernommen, „front desk“ auch auf dem englischen Blatt
Aufschub bleibt „postpone“/„not before“ statt „schedule“ – „frühestens ab“
ist eine Einschränkung, kein Termin.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sessions/Uebersetzung-Gaesteportal-en-2026-10-17.xlsx
+++ b/Sessions/Uebersetzung-Gaesteportal-en-2026-10-17.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Guest portal — sign in</t>
+          <t>Guest portal — Sign in</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>You receive your PIN at check-in.</t>
+          <t>You’ll receive your PIN at check-in.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>We use personal access links: please scan the QR code on the sheet you received at check-in, or open the link in your email. The form below only applies if you received a PIN at check-in.</t>
+          <t>We use individual access links. Please scan the QR code on the sheet you received at check-in, or open the link in your email. Use the form below only if you received a PIN at check-in.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
@@ -983,7 +983,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Please contact reception.</t>
+          <t>Please contact the front desk.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr"/>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>You can also use the property’s web address — it is on the sheet you received at check-in. Reception is always happy to help.</t>
+          <t>Alternatively, you can use the property’s web address, which is printed on the sheet you received at check-in. The front desk will be happy to help.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr"/>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>The access was valid for one stay and expired at check-out. For a new stay, reception will give you new access — they are always happy to help.</t>
+          <t>This access was valid for one stay and expired at check-out. For your next stay, the front desk can provide new access and will be happy to help.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Cleaning is planned.</t>
+          <t>Cleaning is scheduled.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Housekeeping will stop by today.</t>
+          <t>Housekeeping is scheduled to visit today.</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Cleaning today from {time}.</t>
+          <t>Cleaning today, not before {time}.</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr"/>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>We got your request — nobody will come before then.</t>
+          <t>Your request has been noted — no one will come before then.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>As agreed at the door — nobody will come before then.</t>
+          <t>As discussed at your door, no one will come before then.</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>We clean daily. If you don’t need cleaning today, tap “No cleaning today”.</t>
+          <t>We clean daily. If you don’t need your room cleaned today, tap “No cleaning today”.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Today is your day of departure.</t>
+          <t>Today is your check-out day.</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr"/>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>From tomorrow, we clean daily from {time}. Would you like cleaning today already? Tap “Clean my room”.</t>
+          <t>Starting tomorrow, we clean daily from {time}. Would you like your room cleaned today? Tap “Clean my room”.</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr"/>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Housekeeping will come no earlier than {time}</t>
+          <t>Housekeeping will arrive no earlier than {time}</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr"/>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Today, only “now” is still possible.</t>
+          <t>Only “now” is available for the rest of today.</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr"/>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>You can postpone cleaning until &lt;b&gt;{limit}&lt;/b&gt; at the latest — nobody will come before then. We set this limit so that cleaning can still happen the same day.</t>
+          <t>You can postpone cleaning until &lt;b&gt;{limit}&lt;/b&gt; at the latest — no one will come before then. This cutoff helps us make sure your room can still be cleaned today.</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr"/>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>We accept cleaning requests daily between &lt;b&gt;{start}&lt;/b&gt; and &lt;b&gt;{end}&lt;/b&gt;. Simply tap “Clean my room” again during that time — or contact reception.</t>
+          <t>We accept cleaning requests daily between &lt;b&gt;{start}&lt;/b&gt; and &lt;b&gt;{end}&lt;/b&gt;. During those hours, tap “Clean my room” again, or contact the front desk.</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Services still come. Cleaning resumes tomorrow.</t>
+          <t>Other services still come to your room. Cleaning will resume tomorrow.</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr"/>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Nobody knocks — not even for services.</t>
+          <t>No one will knock, including staff delivering other services.</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Reception has your request.</t>
+          <t>The front desk has received your request.</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr"/>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>not provided</t>
+          <t>canceled</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Your stay has ended, and with it your access to the guest portal.</t>
+          <t>Your stay has ended, and your access to the guest portal has expired.</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>We would be delighted if you left a review — it helps other guests choose.</t>
+          <t>We’d appreciate a review. It helps other guests choose where to stay.</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr"/>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Sign-in failed — room number or PIN is incorrect.</t>
+          <t>Sign-in failed — the room number or PIN is incorrect.</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr"/>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Too many failed attempts — please try again in {minutes} min. or contact reception.</t>
+          <t>Too many failed attempts — please try again in {minutes} min. or contact the front desk.</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr"/>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Cleaning requests are only possible between {start} and {end}.</t>
+          <t>You can submit cleaning requests only between {start} and {end}.</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>We don’t offer postponing.</t>
+          <t>Postponing cleaning isn’t available at this property.</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr"/>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Postponing is only possible until {time}.</t>
+          <t>You can postpone cleaning only until {time}.</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr"/>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>We only clean on request.</t>
+          <t>This property offers cleaning on request only.</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr"/>

</xml_diff>